<commit_message>
GBDS MAY FILES 2026 | berlyn@gbds
</commit_message>
<xml_diff>
--- a/GBDS JUNE FILES 2026/CSR MONTH OF JUNE 2026.xlsx
+++ b/GBDS JUNE FILES 2026/CSR MONTH OF JUNE 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS JUNE FILES 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{461A8DE4-79D0-4691-B457-FB7659802252}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B71E35-7E12-40C1-BF2C-3983FAA48276}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="10" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
   </bookViews>
   <sheets>
     <sheet name="CSR | JUNE" sheetId="902" r:id="rId1"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2487" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2499" uniqueCount="92">
   <si>
     <t>CHECKER STOCK REPORT</t>
   </si>
@@ -356,6 +356,18 @@
   </si>
   <si>
     <t>9/3B</t>
+  </si>
+  <si>
+    <t>12B</t>
+  </si>
+  <si>
+    <t>13/12B</t>
+  </si>
+  <si>
+    <t>2/3B</t>
+  </si>
+  <si>
+    <t>12/3B</t>
   </si>
 </sst>
 </file>
@@ -976,7 +988,7 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1223,6 +1235,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3084,47 +3100,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -3356,12 +3372,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -4690,47 +4706,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -4962,12 +4978,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -5003,17 +5019,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -6312,47 +6328,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -6584,12 +6600,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -6625,17 +6641,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7934,47 +7950,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -8206,12 +8222,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -8247,20 +8263,20 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91">
+      <c r="C44" s="92">
         <f>1+1+26+15+15+3+5+62+2+10+551</f>
         <v>691</v>
       </c>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -9557,47 +9573,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -9829,12 +9845,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -11163,47 +11179,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -11435,12 +11451,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -11476,17 +11492,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -12785,47 +12801,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -13057,12 +13073,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -13098,17 +13114,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -14407,47 +14423,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -14679,12 +14695,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -14720,20 +14736,20 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91">
+      <c r="C44" s="92">
         <f>1+1+26+15+15+3+5+62+2+10+551</f>
         <v>691</v>
       </c>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -16030,47 +16046,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -16302,12 +16318,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -17636,47 +17652,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -17908,12 +17924,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -17949,17 +17965,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -19256,47 +19272,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -19528,12 +19544,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -20860,47 +20876,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -21132,12 +21148,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -21173,17 +21189,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -22482,47 +22498,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -22754,12 +22770,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -22795,20 +22811,20 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91">
+      <c r="C44" s="92">
         <f>1+1+26+15+15+3+5+62+2+10+551</f>
         <v>691</v>
       </c>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -24105,47 +24121,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -24377,12 +24393,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -25711,47 +25727,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -25983,12 +25999,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -26024,17 +26040,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -27333,47 +27349,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -27605,12 +27621,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -27646,17 +27662,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -28955,47 +28971,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -29227,12 +29243,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -29268,20 +29284,20 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91">
+      <c r="C44" s="92">
         <f>1+1+26+15+15+3+5+62+2+10+551</f>
         <v>691</v>
       </c>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -30578,47 +30594,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -30850,12 +30866,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -32184,47 +32200,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -32456,12 +32472,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -32497,17 +32513,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -33806,47 +33822,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -34078,12 +34094,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -34119,17 +34135,17 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -35428,47 +35444,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -35700,12 +35716,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -35741,20 +35757,20 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91">
+      <c r="C44" s="92">
         <f>1+1+26+15+15+3+5+62+2+10+551</f>
         <v>691</v>
       </c>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -37116,47 +37132,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -37436,12 +37452,12 @@
       <c r="Q42" s="43">
         <v>19</v>
       </c>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -37477,23 +37493,23 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91">
+      <c r="C44" s="92">
         <f>2+6+10+10+13+10+570</f>
         <v>621</v>
       </c>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91">
+      <c r="C45" s="92">
         <f>22+12+1</f>
         <v>35</v>
       </c>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -38864,47 +38880,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -39176,12 +39192,12 @@
       <c r="Q42" s="43">
         <v>3</v>
       </c>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -39217,22 +39233,22 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91">
+      <c r="C44" s="92">
         <f>1+3+1+1+40+6+275</f>
         <v>327</v>
       </c>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91">
+      <c r="C45" s="92">
         <v>12</v>
       </c>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -40597,47 +40613,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -40905,12 +40921,12 @@
       <c r="Q42" s="43">
         <v>13</v>
       </c>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -40946,20 +40962,20 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91">
+      <c r="C44" s="92">
         <f>10+2+3+1+25+6+307</f>
         <v>354</v>
       </c>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -42256,47 +42272,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -42528,12 +42544,12 @@
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
       <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -42591,7 +42607,8 @@
     <col min="2" max="2" width="14.42578125" style="2" customWidth="1"/>
     <col min="3" max="5" width="5.7109375" style="2" customWidth="1"/>
     <col min="6" max="6" width="8" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="5.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="5.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="7" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="5.7109375" style="2" customWidth="1"/>
@@ -42960,12 +42977,16 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
+      <c r="C8" s="13">
+        <v>2</v>
+      </c>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>79</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -42977,11 +42998,17 @@
       <c r="Q8" s="14"/>
       <c r="R8" s="14"/>
       <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
+      <c r="T8" s="14">
+        <v>1</v>
+      </c>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="59"/>
+      <c r="W8" s="14">
+        <v>1</v>
+      </c>
+      <c r="X8" s="59">
+        <v>1</v>
+      </c>
       <c r="Y8" s="15"/>
     </row>
     <row r="9" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -43148,12 +43175,16 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
+      <c r="C15" s="22">
+        <v>1</v>
+      </c>
       <c r="D15" s="23"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23">
+        <v>11</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -43165,23 +43196,33 @@
       <c r="Q15" s="23"/>
       <c r="R15" s="23"/>
       <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
+      <c r="T15" s="23">
+        <v>1</v>
+      </c>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
-      <c r="X15" s="61"/>
+      <c r="W15" s="23">
+        <v>1</v>
+      </c>
+      <c r="X15" s="61">
+        <v>1</v>
+      </c>
       <c r="Y15" s="24"/>
     </row>
     <row r="16" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="57"/>
+      <c r="C16" s="57">
+        <v>1</v>
+      </c>
       <c r="D16" s="58"/>
       <c r="E16" s="27"/>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
+      <c r="H16" s="28" t="s">
+        <v>88</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="56"/>
@@ -43193,11 +43234,17 @@
       <c r="Q16" s="28"/>
       <c r="R16" s="28"/>
       <c r="S16" s="28"/>
-      <c r="T16" s="28"/>
+      <c r="T16" s="28">
+        <v>0</v>
+      </c>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
-      <c r="X16" s="62"/>
+      <c r="W16" s="56">
+        <v>0</v>
+      </c>
+      <c r="X16" s="62">
+        <v>0</v>
+      </c>
       <c r="Y16" s="29"/>
     </row>
     <row r="17" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -43600,14 +43647,24 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14">
+        <v>2</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>20</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14">
+        <v>1</v>
+      </c>
+      <c r="L24" s="14">
+        <v>10</v>
+      </c>
+      <c r="M24" s="14">
+        <v>341</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
       <c r="P24" s="14"/>
@@ -43786,14 +43843,24 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23">
+        <v>1</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>9</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>1</v>
+      </c>
+      <c r="L31" s="23">
+        <v>8</v>
+      </c>
+      <c r="M31" s="23">
+        <v>37</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
       <c r="P31" s="23"/>
@@ -43814,14 +43881,24 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>1</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>11</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>0</v>
+      </c>
+      <c r="L32" s="28">
+        <v>2</v>
+      </c>
+      <c r="M32" s="28">
+        <v>304</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
       <c r="P32" s="28"/>
@@ -43862,47 +43939,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -43963,19 +44040,35 @@
       </c>
       <c r="C36" s="46"/>
       <c r="D36" s="41"/>
-      <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
+      <c r="E36" s="42">
+        <v>23</v>
+      </c>
+      <c r="F36" s="42">
+        <v>312</v>
+      </c>
+      <c r="G36" s="42">
+        <v>5</v>
+      </c>
       <c r="H36" s="42"/>
-      <c r="I36" s="42"/>
+      <c r="I36" s="42">
+        <v>2</v>
+      </c>
       <c r="J36" s="42"/>
       <c r="K36" s="42"/>
       <c r="L36" s="42"/>
-      <c r="M36" s="42"/>
-      <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
+      <c r="M36" s="42">
+        <v>2</v>
+      </c>
+      <c r="N36" s="42">
+        <v>1</v>
+      </c>
+      <c r="O36" s="42">
+        <v>1</v>
+      </c>
       <c r="P36" s="42"/>
-      <c r="Q36" s="43"/>
+      <c r="Q36" s="43">
+        <v>6</v>
+      </c>
       <c r="R36" s="72"/>
       <c r="S36" s="44"/>
       <c r="T36" s="44"/>
@@ -44121,25 +44214,41 @@
       </c>
       <c r="C42" s="46"/>
       <c r="D42" s="41"/>
-      <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
+      <c r="E42" s="42">
+        <v>23</v>
+      </c>
+      <c r="F42" s="42">
+        <v>312</v>
+      </c>
+      <c r="G42" s="42">
+        <v>5</v>
+      </c>
       <c r="H42" s="42"/>
-      <c r="I42" s="42"/>
+      <c r="I42" s="42">
+        <v>2</v>
+      </c>
       <c r="J42" s="42"/>
       <c r="K42" s="42"/>
       <c r="L42" s="42"/>
-      <c r="M42" s="42"/>
-      <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
+      <c r="M42" s="42">
+        <v>2</v>
+      </c>
+      <c r="N42" s="42">
+        <v>1</v>
+      </c>
+      <c r="O42" s="42">
+        <v>1</v>
+      </c>
       <c r="P42" s="42"/>
-      <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="Q42" s="43">
+        <v>6</v>
+      </c>
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -44175,17 +44284,22 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92">
+        <f>1+1+11+2+304</f>
+        <v>319</v>
+      </c>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92">
+        <v>12</v>
+      </c>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -44213,7 +44327,8 @@
   <cols>
     <col min="1" max="1" width="1.140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="2" customWidth="1"/>
-    <col min="3" max="8" width="5.7109375" style="2" customWidth="1"/>
+    <col min="3" max="7" width="5.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="7" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="13" width="5.7109375" style="2" customWidth="1"/>
@@ -44582,12 +44697,16 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="78"/>
+      <c r="C8" s="80">
+        <v>1</v>
+      </c>
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>89</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -44599,11 +44718,17 @@
       <c r="Q8" s="14"/>
       <c r="R8" s="14"/>
       <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
+      <c r="T8" s="14">
+        <v>1</v>
+      </c>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="59"/>
+      <c r="W8" s="14">
+        <v>2</v>
+      </c>
+      <c r="X8" s="59">
+        <v>1</v>
+      </c>
       <c r="Y8" s="15"/>
     </row>
     <row r="9" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -44770,12 +44895,16 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
+      <c r="C15" s="22">
+        <v>1</v>
+      </c>
       <c r="D15" s="23"/>
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23" t="s">
+        <v>88</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -44787,23 +44916,33 @@
       <c r="Q15" s="23"/>
       <c r="R15" s="23"/>
       <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
+      <c r="T15" s="23">
+        <v>1</v>
+      </c>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
-      <c r="X15" s="61"/>
+      <c r="W15" s="23">
+        <v>2</v>
+      </c>
+      <c r="X15" s="61">
+        <v>1</v>
+      </c>
       <c r="Y15" s="24"/>
     </row>
     <row r="16" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="57"/>
+      <c r="C16" s="57">
+        <v>0</v>
+      </c>
       <c r="D16" s="58"/>
       <c r="E16" s="27"/>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
+      <c r="H16" s="28">
+        <v>13</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="56"/>
@@ -44815,11 +44954,17 @@
       <c r="Q16" s="28"/>
       <c r="R16" s="28"/>
       <c r="S16" s="28"/>
-      <c r="T16" s="28"/>
+      <c r="T16" s="28">
+        <v>0</v>
+      </c>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
-      <c r="X16" s="62"/>
+      <c r="W16" s="56">
+        <v>0</v>
+      </c>
+      <c r="X16" s="62">
+        <v>0</v>
+      </c>
       <c r="Y16" s="29"/>
     </row>
     <row r="17" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -45222,17 +45367,29 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14" t="s">
+        <v>85</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>24</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="L24" s="14">
+        <v>6</v>
+      </c>
+      <c r="M24" s="14">
+        <v>411</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14" t="s">
+        <v>86</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
@@ -45408,17 +45565,29 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23" t="s">
+        <v>88</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>23</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="L31" s="23">
+        <v>6</v>
+      </c>
+      <c r="M31" s="23">
+        <v>81</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23" t="s">
+        <v>86</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
@@ -45436,17 +45605,29 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>1</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>1</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>0</v>
+      </c>
+      <c r="L32" s="28">
+        <v>0</v>
+      </c>
+      <c r="M32" s="28">
+        <v>330</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -45484,47 +45665,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -45583,10 +45764,14 @@
       <c r="B36" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="46"/>
+      <c r="C36" s="46">
+        <v>1</v>
+      </c>
       <c r="D36" s="41"/>
       <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
+      <c r="F36" s="42">
+        <v>334</v>
+      </c>
       <c r="G36" s="42"/>
       <c r="H36" s="42"/>
       <c r="I36" s="42"/>
@@ -45595,9 +45780,15 @@
       <c r="L36" s="42"/>
       <c r="M36" s="42"/>
       <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
-      <c r="P36" s="42"/>
-      <c r="Q36" s="43"/>
+      <c r="O36" s="42">
+        <v>3</v>
+      </c>
+      <c r="P36" s="42">
+        <v>11</v>
+      </c>
+      <c r="Q36" s="43">
+        <v>2</v>
+      </c>
       <c r="R36" s="72"/>
       <c r="S36" s="44"/>
       <c r="T36" s="44"/>
@@ -45741,10 +45932,14 @@
       <c r="B42" s="45" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="46"/>
+      <c r="C42" s="46">
+        <v>1</v>
+      </c>
       <c r="D42" s="41"/>
       <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
+      <c r="F42" s="42">
+        <v>334</v>
+      </c>
       <c r="G42" s="42"/>
       <c r="H42" s="42"/>
       <c r="I42" s="42"/>
@@ -45753,15 +45948,21 @@
       <c r="L42" s="42"/>
       <c r="M42" s="42"/>
       <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
-      <c r="P42" s="42"/>
-      <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="O42" s="42">
+        <v>3</v>
+      </c>
+      <c r="P42" s="42">
+        <v>11</v>
+      </c>
+      <c r="Q42" s="43">
+        <v>2</v>
+      </c>
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -45797,17 +45998,20 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91"/>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92">
+        <f>13+1+1+330</f>
+        <v>345</v>
+      </c>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -46204,29 +46408,63 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
+      <c r="C8" s="13">
+        <v>11</v>
+      </c>
+      <c r="D8" s="14">
+        <v>2</v>
+      </c>
+      <c r="E8" s="14">
+        <v>5</v>
+      </c>
+      <c r="F8" s="14">
+        <v>2</v>
+      </c>
+      <c r="G8" s="14">
+        <v>5</v>
+      </c>
+      <c r="H8" s="14">
+        <v>5</v>
+      </c>
+      <c r="I8" s="14">
+        <v>1</v>
+      </c>
       <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
+      <c r="K8" s="14">
+        <v>1</v>
+      </c>
       <c r="L8" s="14"/>
       <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
+      <c r="N8" s="14">
+        <v>1</v>
+      </c>
+      <c r="O8" s="14">
+        <v>1</v>
+      </c>
+      <c r="P8" s="14">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="14">
+        <v>1</v>
+      </c>
       <c r="R8" s="14"/>
-      <c r="S8" s="14"/>
+      <c r="S8" s="14">
+        <v>1</v>
+      </c>
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
-      <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="59"/>
-      <c r="Y8" s="15"/>
+      <c r="V8" s="14">
+        <v>2</v>
+      </c>
+      <c r="W8" s="14">
+        <v>10</v>
+      </c>
+      <c r="X8" s="59">
+        <v>10</v>
+      </c>
+      <c r="Y8" s="15">
+        <v>2</v>
+      </c>
     </row>
     <row r="9" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
@@ -46392,57 +46630,125 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
+      <c r="C15" s="22">
+        <v>1</v>
+      </c>
+      <c r="D15" s="23">
+        <v>2</v>
+      </c>
+      <c r="E15" s="23">
+        <v>0</v>
+      </c>
+      <c r="F15" s="23">
+        <v>0</v>
+      </c>
+      <c r="G15" s="23">
+        <v>0</v>
+      </c>
+      <c r="H15" s="23">
+        <v>4</v>
+      </c>
+      <c r="I15" s="23">
+        <v>0</v>
+      </c>
       <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
+      <c r="K15" s="23">
+        <v>0</v>
+      </c>
       <c r="L15" s="23"/>
       <c r="M15" s="23"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="23"/>
-      <c r="P15" s="23"/>
-      <c r="Q15" s="23"/>
+      <c r="N15" s="23">
+        <v>0</v>
+      </c>
+      <c r="O15" s="23">
+        <v>0</v>
+      </c>
+      <c r="P15" s="23">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="23">
+        <v>0</v>
+      </c>
       <c r="R15" s="23"/>
-      <c r="S15" s="23"/>
+      <c r="S15" s="23">
+        <v>0</v>
+      </c>
       <c r="T15" s="23"/>
       <c r="U15" s="23"/>
-      <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
-      <c r="X15" s="61"/>
-      <c r="Y15" s="24"/>
+      <c r="V15" s="23">
+        <v>0</v>
+      </c>
+      <c r="W15" s="23">
+        <v>0</v>
+      </c>
+      <c r="X15" s="61">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="24">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="57"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
-      <c r="I16" s="28"/>
+      <c r="C16" s="57">
+        <v>10</v>
+      </c>
+      <c r="D16" s="58">
+        <v>0</v>
+      </c>
+      <c r="E16" s="27">
+        <v>5</v>
+      </c>
+      <c r="F16" s="27">
+        <v>2</v>
+      </c>
+      <c r="G16" s="28">
+        <v>5</v>
+      </c>
+      <c r="H16" s="28">
+        <v>1</v>
+      </c>
+      <c r="I16" s="28">
+        <v>1</v>
+      </c>
       <c r="J16" s="28"/>
-      <c r="K16" s="56"/>
+      <c r="K16" s="56">
+        <v>1</v>
+      </c>
       <c r="L16" s="28"/>
       <c r="M16" s="28"/>
-      <c r="N16" s="28"/>
-      <c r="O16" s="28"/>
-      <c r="P16" s="28"/>
-      <c r="Q16" s="28"/>
+      <c r="N16" s="28">
+        <v>1</v>
+      </c>
+      <c r="O16" s="28">
+        <v>1</v>
+      </c>
+      <c r="P16" s="28">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="28">
+        <v>1</v>
+      </c>
       <c r="R16" s="28"/>
-      <c r="S16" s="28"/>
+      <c r="S16" s="28">
+        <v>1</v>
+      </c>
       <c r="T16" s="28"/>
       <c r="U16" s="28"/>
-      <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
-      <c r="X16" s="62"/>
-      <c r="Y16" s="29"/>
+      <c r="V16" s="28">
+        <v>2</v>
+      </c>
+      <c r="W16" s="56">
+        <v>10</v>
+      </c>
+      <c r="X16" s="62">
+        <v>10</v>
+      </c>
+      <c r="Y16" s="29">
+        <v>2</v>
+      </c>
     </row>
     <row r="17" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="30"/>
@@ -46842,25 +47148,51 @@
         <v>23</v>
       </c>
       <c r="C24" s="13"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="D24" s="14">
+        <v>2</v>
+      </c>
+      <c r="E24" s="14">
+        <v>2</v>
+      </c>
+      <c r="F24" s="14">
+        <v>7</v>
+      </c>
+      <c r="G24" s="14">
+        <v>1</v>
+      </c>
+      <c r="H24" s="14">
+        <v>102</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="14"/>
+      <c r="K24" s="14">
+        <v>1</v>
+      </c>
+      <c r="L24" s="14">
+        <v>20</v>
+      </c>
+      <c r="M24" s="14">
+        <v>348</v>
+      </c>
+      <c r="N24" s="14">
+        <v>1</v>
+      </c>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14" t="s">
+        <v>91</v>
+      </c>
       <c r="Q24" s="14"/>
-      <c r="R24" s="14"/>
+      <c r="R24" s="14">
+        <v>1</v>
+      </c>
       <c r="S24" s="14"/>
       <c r="T24" s="14"/>
-      <c r="U24" s="14"/>
-      <c r="V24" s="14"/>
+      <c r="U24" s="14">
+        <v>1</v>
+      </c>
+      <c r="V24" s="14">
+        <v>1</v>
+      </c>
       <c r="W24" s="14"/>
       <c r="X24" s="14"/>
       <c r="Y24" s="15"/>
@@ -47028,25 +47360,51 @@
         <v>25</v>
       </c>
       <c r="C31" s="22"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="D31" s="23">
+        <v>0</v>
+      </c>
+      <c r="E31" s="23">
+        <v>0</v>
+      </c>
+      <c r="F31" s="23">
+        <v>7</v>
+      </c>
+      <c r="G31" s="23">
+        <v>0</v>
+      </c>
+      <c r="H31" s="23">
+        <v>28</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
-      <c r="N31" s="23"/>
+      <c r="K31" s="23">
+        <v>0</v>
+      </c>
+      <c r="L31" s="23">
+        <v>0</v>
+      </c>
+      <c r="M31" s="23">
+        <v>2</v>
+      </c>
+      <c r="N31" s="23">
+        <v>0</v>
+      </c>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23" t="s">
+        <v>90</v>
+      </c>
       <c r="Q31" s="23"/>
-      <c r="R31" s="23"/>
+      <c r="R31" s="23">
+        <v>0</v>
+      </c>
       <c r="S31" s="23"/>
       <c r="T31" s="23"/>
-      <c r="U31" s="23"/>
-      <c r="V31" s="23"/>
+      <c r="U31" s="23">
+        <v>0</v>
+      </c>
+      <c r="V31" s="23">
+        <v>0</v>
+      </c>
       <c r="W31" s="23"/>
       <c r="X31" s="61"/>
       <c r="Y31" s="24"/>
@@ -47056,25 +47414,51 @@
         <v>26</v>
       </c>
       <c r="C32" s="26"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="D32" s="27">
+        <v>2</v>
+      </c>
+      <c r="E32" s="27">
+        <v>2</v>
+      </c>
+      <c r="F32" s="27">
+        <v>0</v>
+      </c>
+      <c r="G32" s="28">
+        <v>1</v>
+      </c>
+      <c r="H32" s="28">
+        <v>74</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="28"/>
+      <c r="K32" s="28">
+        <v>1</v>
+      </c>
+      <c r="L32" s="28">
+        <v>20</v>
+      </c>
+      <c r="M32" s="28">
+        <v>346</v>
+      </c>
+      <c r="N32" s="28">
+        <v>1</v>
+      </c>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>10</v>
+      </c>
       <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
+      <c r="R32" s="28">
+        <v>1</v>
+      </c>
       <c r="S32" s="28"/>
       <c r="T32" s="28"/>
-      <c r="U32" s="28"/>
-      <c r="V32" s="28"/>
+      <c r="U32" s="28">
+        <v>1</v>
+      </c>
+      <c r="V32" s="28">
+        <v>1</v>
+      </c>
       <c r="W32" s="28"/>
       <c r="X32" s="63"/>
       <c r="Y32" s="29"/>
@@ -47106,47 +47490,47 @@
       <c r="Y33" s="31"/>
     </row>
     <row r="34" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="87" t="s">
+      <c r="C34" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="87"/>
-      <c r="E34" s="88"/>
-      <c r="F34" s="89" t="s">
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="90" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="87"/>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89" t="s">
+      <c r="G34" s="88"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="J34" s="87"/>
-      <c r="K34" s="88"/>
-      <c r="L34" s="89" t="s">
+      <c r="J34" s="88"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="90" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="87"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="90" t="s">
+      <c r="M34" s="88"/>
+      <c r="N34" s="89"/>
+      <c r="O34" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="90"/>
-      <c r="R34" s="80" t="s">
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+      <c r="R34" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="82"/>
+      <c r="S34" s="82"/>
+      <c r="T34" s="82"/>
+      <c r="U34" s="83"/>
       <c r="V34" s="66"/>
       <c r="W34" s="3"/>
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
     <row r="35" spans="2:25" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="86"/>
+      <c r="B35" s="87"/>
       <c r="C35" s="50" t="s">
         <v>49</v>
       </c>
@@ -47205,21 +47589,45 @@
       <c r="B36" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="46"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
-      <c r="H36" s="42"/>
+      <c r="C36" s="46">
+        <v>1</v>
+      </c>
+      <c r="D36" s="41">
+        <v>7</v>
+      </c>
+      <c r="E36" s="42">
+        <v>11</v>
+      </c>
+      <c r="F36" s="42">
+        <v>278</v>
+      </c>
+      <c r="G36" s="42">
+        <v>382</v>
+      </c>
+      <c r="H36" s="42">
+        <v>5</v>
+      </c>
       <c r="I36" s="42"/>
-      <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
-      <c r="M36" s="42"/>
-      <c r="N36" s="42"/>
+      <c r="J36" s="42">
+        <v>32</v>
+      </c>
+      <c r="K36" s="42">
+        <v>7</v>
+      </c>
+      <c r="L36" s="42">
+        <v>3</v>
+      </c>
+      <c r="M36" s="42">
+        <v>69</v>
+      </c>
+      <c r="N36" s="42">
+        <v>10</v>
+      </c>
       <c r="O36" s="42"/>
       <c r="P36" s="42"/>
-      <c r="Q36" s="43"/>
+      <c r="Q36" s="43">
+        <v>5</v>
+      </c>
       <c r="R36" s="72"/>
       <c r="S36" s="44"/>
       <c r="T36" s="44"/>
@@ -47363,27 +47771,51 @@
       <c r="B42" s="45" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="46"/>
-      <c r="D42" s="41"/>
-      <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
-      <c r="H42" s="42"/>
+      <c r="C42" s="46">
+        <v>1</v>
+      </c>
+      <c r="D42" s="41">
+        <v>7</v>
+      </c>
+      <c r="E42" s="42">
+        <v>11</v>
+      </c>
+      <c r="F42" s="42">
+        <v>278</v>
+      </c>
+      <c r="G42" s="42">
+        <v>382</v>
+      </c>
+      <c r="H42" s="42">
+        <v>5</v>
+      </c>
       <c r="I42" s="42"/>
-      <c r="J42" s="42"/>
-      <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
-      <c r="M42" s="42"/>
-      <c r="N42" s="42"/>
+      <c r="J42" s="42">
+        <v>32</v>
+      </c>
+      <c r="K42" s="42">
+        <v>7</v>
+      </c>
+      <c r="L42" s="42">
+        <v>3</v>
+      </c>
+      <c r="M42" s="42">
+        <v>69</v>
+      </c>
+      <c r="N42" s="42">
+        <v>10</v>
+      </c>
       <c r="O42" s="42"/>
       <c r="P42" s="42"/>
-      <c r="Q42" s="43"/>
-      <c r="R42" s="83" t="s">
+      <c r="Q42" s="43">
+        <v>5</v>
+      </c>
+      <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="S42" s="84"/>
-      <c r="T42" s="84"/>
-      <c r="U42" s="84"/>
+      <c r="S42" s="85"/>
+      <c r="T42" s="85"/>
+      <c r="U42" s="85"/>
       <c r="V42" s="3"/>
       <c r="W42" s="3"/>
       <c r="X42" s="3"/>
@@ -47419,20 +47851,20 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="91">
-        <f>1+1+26+15+15+3+5+62+2+10+551</f>
-        <v>691</v>
-      </c>
-      <c r="D44" s="91"/>
-      <c r="E44" s="91"/>
+      <c r="C44" s="92">
+        <f>10+5+2+5+1+1+1+1+1+1+1+1+2+10+10+2+2+2+1+74+1+20+346+1+10+1+1+1</f>
+        <v>514</v>
+      </c>
+      <c r="D44" s="92"/>
+      <c r="E44" s="92"/>
     </row>
     <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
+      <c r="C45" s="92"/>
+      <c r="D45" s="92"/>
+      <c r="E45" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
GBDS JUNE FILES 2026 | berlyn@gbds
</commit_message>
<xml_diff>
--- a/GBDS JUNE FILES 2026/CSR MONTH OF JUNE 2026.xlsx
+++ b/GBDS JUNE FILES 2026/CSR MONTH OF JUNE 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS JUNE FILES 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B71E35-7E12-40C1-BF2C-3983FAA48276}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E10AB9-7614-4FC3-B0C0-FF1CA00911D8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="10" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="8" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
   </bookViews>
   <sheets>
     <sheet name="CSR | JUNE" sheetId="902" r:id="rId1"/>

</xml_diff>